<commit_message>
docs: add unedited walkthrough and edited showcase video links across submission docs
</commit_message>
<xml_diff>
--- a/Assessment3_Lakshmandev_Vk.xlsx
+++ b/Assessment3_Lakshmandev_Vk.xlsx
@@ -519,7 +519,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="96" customWidth="1" min="2" max="2"/>
@@ -720,7 +720,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
@@ -854,7 +854,8 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>[Insert your unedited Loom / Google Drive link here before submitting email]</t>
+          <t>https://drive.google.com/file/d/1DMZmS_t_iJfAsIb9ll3Qhc8AiPU1lksB/view?usp=sharing
+(Edited Version: https://drive.google.com/file/d/1E7Qa8Tcy89PY3jZ7xDU9TJP4RTOZsFnl/view?usp=sharing)</t>
         </is>
       </c>
     </row>
@@ -939,7 +940,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
@@ -1258,7 +1259,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
@@ -1673,7 +1674,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
@@ -1989,7 +1990,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
@@ -2254,7 +2255,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
@@ -2534,7 +2535,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
docs: clarify unedited vs edited demo video URLs in Excel workbook
</commit_message>
<xml_diff>
--- a/Assessment3_Lakshmandev_Vk.xlsx
+++ b/Assessment3_Lakshmandev_Vk.xlsx
@@ -846,7 +846,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="28.2" customHeight="1">
+    <row r="13" ht="58" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Demo video URL (max 8 min, unedited)</t>
@@ -854,8 +854,10 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1DMZmS_t_iJfAsIb9ll3Qhc8AiPU1lksB/view?usp=sharing
-(Edited Version: https://drive.google.com/file/d/1E7Qa8Tcy89PY3jZ7xDU9TJP4RTOZsFnl/view?usp=sharing)</t>
+          <t>Unedited Video (Official Walkthrough, max 8 min):
+https://drive.google.com/file/d/1DMZmS_t_iJfAsIb9ll3Qhc8AiPU1lksB/view?usp=sharing
+Edited Video (Showcase):
+https://drive.google.com/file/d/1E7Qa8Tcy89PY3jZ7xDU9TJP4RTOZsFnl/view?usp=sharing</t>
         </is>
       </c>
     </row>

</xml_diff>